<commit_message>
Fixed county cleaning resulting in low outer island data and fixed paths in prepare_data and app
</commit_message>
<xml_diff>
--- a/data/Analytic Code Output/Missing_Coordinates.xlsx
+++ b/data/Analytic Code Output/Missing_Coordinates.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -371,6 +371,79 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MORTLOCK</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MORTLOCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MORTLOCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NORTHWEST</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NORTHWEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NORTHWEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UTWE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ZZ-UNKNOWN-CHUUK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ZZ-UNKNOWN-KOSRAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ZZ-UNKNOWN-POHNPEI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ZZ-UNKNOWN-YAP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>